<commit_message>
Updated GRC model - 2025-09-13 00:19
</commit_message>
<xml_diff>
--- a/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GRC\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8553E8F-21CD-41DB-94EA-C97D2338D234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{11CF31A6-7C9B-4F7D-9615-3EC86D49F829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7536,7 +7536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD44996E-6E9D-40EB-91B9-24874ED1BEA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65A19E21-FC76-44C1-94CF-92FB711CEF2A}">
   <dimension ref="B9:N40"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8732,7 +8732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74687C68-8BAF-4F13-8566-7F68B3E26DAC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D11F1047-8240-4188-B61D-9C7ECD4FDE87}">
   <dimension ref="B9:AB165"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19436,7 +19436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7B42E1-F927-4CB0-BCDF-22FD34A5E4C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB820F8A-34E5-49FF-8E09-B8D0E9D98293}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GRC model - 2025-09-13 00:34
</commit_message>
<xml_diff>
--- a/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GRC\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11CF31A6-7C9B-4F7D-9615-3EC86D49F829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E06BB71C-E388-4EC1-B58F-1D408CAAC33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7536,7 +7536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65A19E21-FC76-44C1-94CF-92FB711CEF2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B5376D-6A87-493A-8237-72C9B505F87E}">
   <dimension ref="B9:N40"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8732,7 +8732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D11F1047-8240-4188-B61D-9C7ECD4FDE87}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63EFDEA-3A7F-4B79-89EA-C085F30112D7}">
   <dimension ref="B9:AB165"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19436,7 +19436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB820F8A-34E5-49FF-8E09-B8D0E9D98293}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C3E1A2-7564-4FC5-A622-588025455865}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GRC model - 2025-09-13 00:41
</commit_message>
<xml_diff>
--- a/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GRC\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E06BB71C-E388-4EC1-B58F-1D408CAAC33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BCD45EF-A0E6-4364-9918-A17660FF7BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7536,7 +7536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B5376D-6A87-493A-8237-72C9B505F87E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B32CD22-A9AC-46AF-8F28-3E1B25C35579}">
   <dimension ref="B9:N40"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8732,7 +8732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63EFDEA-3A7F-4B79-89EA-C085F30112D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DFCC6E-06AB-4ECC-A521-E5EE472F98EA}">
   <dimension ref="B9:AB165"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19436,7 +19436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C3E1A2-7564-4FC5-A622-588025455865}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C84177F-14D1-4B7F-BDD7-A14A2E5808FE}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GRC model - 2025-09-13 02:02
</commit_message>
<xml_diff>
--- a/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GRC\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BCD45EF-A0E6-4364-9918-A17660FF7BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB50DA2D-856F-445C-B39B-8880E30489D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7536,7 +7536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B32CD22-A9AC-46AF-8F28-3E1B25C35579}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD128397-A77F-44E9-90EE-7F4C01E8D34A}">
   <dimension ref="B9:N40"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8732,7 +8732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DFCC6E-06AB-4ECC-A521-E5EE472F98EA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919F6CB7-2F94-445E-A4C1-3DE967424F95}">
   <dimension ref="B9:AB165"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19436,7 +19436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C84177F-14D1-4B7F-BDD7-A14A2E5808FE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E0452A-E8AA-429B-BA6B-DA6174CE8DF1}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GRC model - 2025-09-13 09:25
</commit_message>
<xml_diff>
--- a/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GRC\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB50DA2D-856F-445C-B39B-8880E30489D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1602E422-0817-4C3A-9A8D-F1B91D8BD2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7536,7 +7536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD128397-A77F-44E9-90EE-7F4C01E8D34A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D34DB4-923C-49E3-9C9B-6AFB9ABC6D19}">
   <dimension ref="B9:N40"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8732,7 +8732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919F6CB7-2F94-445E-A4C1-3DE967424F95}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4FA977-A16E-49A9-A4E3-323EEF154B30}">
   <dimension ref="B9:AB165"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19436,7 +19436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E0452A-E8AA-429B-BA6B-DA6174CE8DF1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CBCE278-5D75-421E-B3F5-92D82BEBC85F}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GRC model - 2025-09-13 10:06
</commit_message>
<xml_diff>
--- a/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GRC/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GRC\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1602E422-0817-4C3A-9A8D-F1B91D8BD2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDC84D25-12CA-450D-BD3E-85883E6FBB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7536,7 +7536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D34DB4-923C-49E3-9C9B-6AFB9ABC6D19}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF279CAE-C83E-4FE5-9D20-9798170F6F03}">
   <dimension ref="B9:N40"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8732,7 +8732,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4FA977-A16E-49A9-A4E3-323EEF154B30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AE96C14-86A5-4B28-8C6E-04E8C6C4AE6B}">
   <dimension ref="B9:AB165"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -19436,7 +19436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CBCE278-5D75-421E-B3F5-92D82BEBC85F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8FED2AD-7451-49F3-AB84-3CB1833EAF7D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>